<commit_message>
Test file and excel
</commit_message>
<xml_diff>
--- a/results/tables/MAIN TABLE/Gowalla_train/Comparsion.xlsx
+++ b/results/tables/MAIN TABLE/Gowalla_train/Comparsion.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\SEM-6\ELECTIVES\DEPARTMENT-ELECTIVES\Recommendation Systems\RS-Project\results\tables\MAIN TABLE\Gowalla_train\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1535BCC1-28EC-40F0-8EDE-F1C6EBC1DF25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{934CC74E-02C8-42BC-9070-8D37C5EEE053}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,16 +42,16 @@
     <t>4 Layers</t>
   </si>
   <si>
-    <t>Paper Recall@20</t>
-  </si>
-  <si>
-    <t>Paper NDCG@20</t>
-  </si>
-  <si>
-    <t>My Recall@20</t>
-  </si>
-  <si>
-    <t>My NDCG@20</t>
+    <t>My Recall@20(train set)</t>
+  </si>
+  <si>
+    <t>My NDCG@20(train set)</t>
+  </si>
+  <si>
+    <t>Paper Recall@20(test set)</t>
+  </si>
+  <si>
+    <t>Paper NDCG@20(test set)</t>
   </si>
 </sst>
 </file>
@@ -388,26 +388,26 @@
   <cols>
     <col min="1" max="1" width="7.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.21875" customWidth="1"/>
-    <col min="3" max="3" width="14.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.77734375" customWidth="1"/>
     <col min="4" max="4" width="9.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="14.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>7</v>
-      </c>
       <c r="D1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>6</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">

</xml_diff>